<commit_message>
data: publish 2026-10-16 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-16-182路.xlsx
+++ b/data/export/2026-10-16-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -632,32 +632,36 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>78分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -665,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -689,33 +693,37 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>4/13</t>
         </is>
       </c>
     </row>
@@ -743,32 +751,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>77分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -776,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,17 +812,17 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -820,13 +832,17 @@
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>77.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -854,32 +870,36 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>75分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -887,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -911,33 +931,37 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>1/13</t>
         </is>
       </c>
     </row>
@@ -965,32 +989,36 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:52</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>77分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -998,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1022,17 +1050,17 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
@@ -1042,13 +1070,17 @@
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB5" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>77.0</t>
+        </is>
+      </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1141,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1148,7 +1180,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
@@ -1159,7 +1191,7 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1252,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1302,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1363,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1413,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1474,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1492,7 +1524,7 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1500,22 +1532,22 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>沪A67983D</t>
+          <t>沪A68397D</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>07:15</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1548,12 +1580,12 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1567,7 +1599,7 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
@@ -1603,7 +1635,792 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>4/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A02126A</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>1/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-16 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-16-182路.xlsx
+++ b/data/export/2026-10-16-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC17"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>4/13</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -761,12 +761,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>77分钟</t>
+          <t>78分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -827,22 +827,22 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>78.0</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>2/13</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -880,12 +880,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:38</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>75分钟</t>
+          <t>78分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -956,12 +956,12 @@
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>78.0</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>1/13</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -999,24 +999,24 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>07:52</t>
+          <t>07:57</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>77分钟</t>
+          <t>82分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1065,22 +1065,22 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA5" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>82.0</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>2/13</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1108,32 +1108,36 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>81分钟</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1141,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1165,17 +1169,17 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr">
@@ -1185,13 +1189,17 @@
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB6" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>81.0</t>
+        </is>
+      </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -1219,32 +1227,36 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:13</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>85分钟</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
           <t>06:11</t>
@@ -1252,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1276,33 +1288,37 @@
       </c>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA7" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr">
+        <is>
+          <t>85.0</t>
+        </is>
+      </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>7/14</t>
         </is>
       </c>
     </row>
@@ -1330,32 +1346,36 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:18</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>83分钟</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1363,7 +1383,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1387,33 +1407,37 @@
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA8" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="inlineStr">
+        <is>
+          <t>83.0</t>
+        </is>
+      </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -1441,32 +1465,36 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:31</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>91分钟</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
           <t>06:22</t>
@@ -1474,7 +1502,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1498,33 +1526,37 @@
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA9" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB9" s="2" t="inlineStr"/>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>91.0</t>
+        </is>
+      </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1617,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1635,7 +1667,7 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>—/14</t>
         </is>
       </c>
     </row>
@@ -1663,32 +1695,36 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:46</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>91分钟</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1696,7 +1732,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1720,17 +1756,17 @@
       </c>
       <c r="W11" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
@@ -1740,13 +1776,17 @@
       </c>
       <c r="AA11" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB11" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>91.0</t>
+        </is>
+      </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1847,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1857,7 +1897,7 @@
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>—/14</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1958,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1972,7 +2012,7 @@
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>4/13</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2073,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2083,7 +2123,7 @@
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>—/14</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2184,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2194,7 +2234,7 @@
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>—/14</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2295,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2304,12 +2344,12 @@
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>78.0</t>
         </is>
       </c>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>1/13</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -2317,22 +2357,22 @@
       <c r="A17" s="2" t="inlineStr"/>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>沪A67026D</t>
+          <t>沪A66513D</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>08:15</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -2370,7 +2410,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>07:22</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2384,43 +2424,733 @@
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr">
         <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>1/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
           <t>08:15</t>
         </is>
       </c>
-      <c r="V17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>08:12</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr"/>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V18" s="2" t="inlineStr">
         <is>
           <t>计划发车</t>
         </is>
       </c>
-      <c r="W17" s="2" t="inlineStr">
+      <c r="W18" s="2" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X17" s="2" t="inlineStr">
-        <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="Y17" s="2" t="inlineStr">
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="Z17" s="2" t="inlineStr">
+      <c r="Z18" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA17" s="2" t="inlineStr">
+      <c r="AA18" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>82.0</t>
+        </is>
+      </c>
+      <c r="AC18" s="2" t="inlineStr">
+        <is>
+          <t>5/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>08:12</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y19" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z19" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA19" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB19" s="2" t="inlineStr">
+        <is>
+          <t>81.0</t>
+        </is>
+      </c>
+      <c r="AC19" s="2" t="inlineStr">
+        <is>
+          <t>4/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>沪A08953A</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>08:31</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>08:12</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>08:31</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA20" s="2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AB17" s="2" t="inlineStr"/>
-      <c r="AC17" s="2" t="inlineStr">
-        <is>
-          <t>—/13</t>
+      <c r="AB20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="inlineStr">
+        <is>
+          <t>—/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>08:35</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>08:12</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="inlineStr"/>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>08:35</t>
+        </is>
+      </c>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z21" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA21" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB21" s="2" t="inlineStr">
+        <is>
+          <t>85.0</t>
+        </is>
+      </c>
+      <c r="AC21" s="2" t="inlineStr">
+        <is>
+          <t>7/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr"/>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>08:12</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr"/>
+      <c r="T22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z22" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA22" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB22" s="2" t="inlineStr">
+        <is>
+          <t>83.0</t>
+        </is>
+      </c>
+      <c r="AC22" s="2" t="inlineStr">
+        <is>
+          <t>6/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>沪A12050A</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>08:55</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>06:22</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>08:12</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="inlineStr"/>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>08:55</t>
+        </is>
+      </c>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z23" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB23" s="2" t="inlineStr">
+        <is>
+          <t>91.0</t>
+        </is>
+      </c>
+      <c r="AC23" s="2" t="inlineStr">
+        <is>
+          <t>8/14</t>
         </is>
       </c>
     </row>

</xml_diff>